<commit_message>
feat: fix calculate_total_parking_fee task
</commit_message>
<xml_diff>
--- a/packages/surfgym-task/src/surfgym_task/data/spreadsheet/reference/calculate_total_parking_fee/calculate_total_parking_fee_gold.xlsx
+++ b/packages/surfgym-task/src/surfgym_task/data/spreadsheet/reference/calculate_total_parking_fee/calculate_total_parking_fee_gold.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/goonco/01_workspace/09_llm-lab/cua-boot/surfgym/packages/surfgym-task/src/surfgym_task/data/spreadsheet/reference/357ef137-7eeb-4c80-a3bb-0951f26a8aff/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/goonco/01_workspace/09_llm-lab/cua-boot/surfgym/packages/surfgym-task/src/surfgym_task/data/spreadsheet/reference/calculate_total_parking_fee/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B20581-BA2A-0C45-B609-1EBFF7FCACF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06DFF266-C53A-AA41-B072-FEF26DF78E10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="27660" windowHeight="13180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -44,10 +44,11 @@
     <t>Total Hours</t>
   </si>
   <si>
-    <t>Total Earned</t>
+    <t>Hourly Rate</t>
   </si>
   <si>
-    <t>Hourly Rate</t>
+    <t>Total Parking Fee</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -85,6 +86,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="思源黑体 CN Normal"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="8"/>
@@ -698,38 +700,38 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>3</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" s="4">
-        <v>0.100694444444444</v>
+        <v>5.5555555555555552E-2</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="4">
         <f>SUM(B3:B7)</f>
-        <v>0.31944444444444398</v>
+        <v>0.38194444444444442</v>
       </c>
       <c r="E3" s="4">
         <f>D3*24*F3</f>
-        <v>191.66666666666637</v>
+        <v>41.25</v>
       </c>
       <c r="F3" s="7">
-        <v>25</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="4">
-        <v>6.25E-2</v>
+        <v>9.0277777777777776E-2</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -741,7 +743,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="4">
-        <v>3.125E-2</v>
+        <v>3.4722222222222224E-2</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -750,10 +752,10 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" s="4">
-        <v>4.8611111111111098E-2</v>
+        <v>0.13541666666666666</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -762,10 +764,10 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B7" s="4">
-        <v>7.6388888888888895E-2</v>
+        <v>6.5972222222222224E-2</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>

</xml_diff>